<commit_message>
Oatside report: publish reports/oatside-pg-2026 (remove legacy oatside-apr2026) 2026-05-26 13:09
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
+++ b/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer_Trips_Per_Day" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Customer_Trips_Per_Day" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer_Trips_Per_Day'!$A$4:$F$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer_Trips_Per_Day'!$A$4:$F$30</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-09 00:22</t>
+          <t>2026-05-26 13:09</t>
         </is>
       </c>
     </row>
@@ -540,10 +540,10 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46121</v>
+        <v>46143</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>2</v>
@@ -554,13 +554,13 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>46122</v>
+        <v>46144</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D6" s="8" t="n"/>
       <c r="E6" s="8" t="n"/>
@@ -568,13 +568,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46123</v>
+        <v>46145</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
@@ -582,13 +582,13 @@
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>46124</v>
+        <v>46146</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
@@ -596,13 +596,13 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46125</v>
+        <v>46147</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
@@ -610,13 +610,13 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>46126</v>
+        <v>46148</v>
       </c>
       <c r="B10" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
@@ -624,13 +624,13 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46127</v>
+        <v>46149</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
@@ -638,13 +638,13 @@
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>46128</v>
+        <v>46150</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D12" s="8" t="n"/>
       <c r="E12" s="8" t="n"/>
@@ -652,13 +652,13 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>46129</v>
+        <v>46151</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
@@ -666,10 +666,10 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
-        <v>46130</v>
+        <v>46152</v>
       </c>
       <c r="B14" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>3</v>
@@ -680,13 +680,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46131</v>
+        <v>46153</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
@@ -694,13 +694,13 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>46132</v>
+        <v>46154</v>
       </c>
       <c r="B16" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
@@ -708,13 +708,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46133</v>
+        <v>46155</v>
       </c>
       <c r="B17" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
@@ -722,10 +722,10 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>46134</v>
+        <v>46156</v>
       </c>
       <c r="B18" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>4</v>
@@ -736,13 +736,13 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>46135</v>
+        <v>46157</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
@@ -750,13 +750,13 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
-        <v>46137</v>
+        <v>46158</v>
       </c>
       <c r="B20" s="8" t="n">
         <v>3</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
@@ -764,13 +764,13 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>46138</v>
+        <v>46159</v>
       </c>
       <c r="B21" s="6" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
@@ -778,13 +778,13 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>46141</v>
+        <v>46160</v>
       </c>
       <c r="B22" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
@@ -792,20 +792,118 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>46142</v>
+        <v>46161</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D23" s="6" t="n"/>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
     </row>
+    <row r="24">
+      <c r="A24" s="7" t="n">
+        <v>46162</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C25" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="n">
+        <v>46164</v>
+      </c>
+      <c r="B26" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46165</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C27" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B28" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C28" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>46167</v>
+      </c>
+      <c r="B29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="n">
+        <v>46168</v>
+      </c>
+      <c r="B30" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F23"/>
+  <autoFilter ref="A4:F30"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Oatside report: publish reports/oatside-pg-2026 2026-06-05 14:30
- Base 6,400 @ 31.00-31.99 linear 1.5%/baht
- No-work May 1 removed
- Diesel May 30 = 40.70
- 154 trips, 22 unmatched

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
+++ b/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Customer_Trips_Per_Day" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer_Trips_Per_Day'!$A$4:$F$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Customer_Trips_Per_Day'!$A$4:$F$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -506,7 +506,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-05-26 13:20</t>
+          <t>2026-06-05 16:06</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
         <v>46168</v>
       </c>
       <c r="B30" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C30" s="8" t="n">
         <v>4</v>
@@ -902,8 +902,78 @@
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="8" t="n"/>
     </row>
+    <row r="31">
+      <c r="A31" s="5" t="n">
+        <v>46169</v>
+      </c>
+      <c r="B31" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="C33" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n">
+        <v>46173</v>
+      </c>
+      <c r="B35" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C35" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:F30"/>
+  <autoFilter ref="A4:F35"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Oatside report: July 2026 billing (grand 1,537,168 / 184 trips + 25 BH)
</commit_message>
<xml_diff>
--- a/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
+++ b/reports/oatside-pg-2026/exports/01_CPD_MatchedTripsPerDay.xlsx
@@ -506,7 +506,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-06-10 18:21</t>
+          <t>2026-08-04 14:01</t>
         </is>
       </c>
     </row>
@@ -540,13 +540,13 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>46143</v>
+        <v>46204</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
@@ -554,13 +554,13 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>46144</v>
+        <v>46205</v>
       </c>
       <c r="B6" s="8" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D6" s="8" t="n"/>
       <c r="E6" s="8" t="n"/>
@@ -568,13 +568,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>46145</v>
+        <v>46206</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
@@ -582,13 +582,13 @@
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>46146</v>
+        <v>46207</v>
       </c>
       <c r="B8" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
@@ -596,13 +596,13 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="n">
-        <v>46147</v>
+        <v>46208</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
@@ -610,13 +610,13 @@
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>46148</v>
+        <v>46209</v>
       </c>
       <c r="B10" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
@@ -624,13 +624,13 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>46149</v>
+        <v>46210</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D11" s="6" t="n"/>
       <c r="E11" s="6" t="n"/>
@@ -638,13 +638,13 @@
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>46150</v>
+        <v>46211</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D12" s="8" t="n"/>
       <c r="E12" s="8" t="n"/>
@@ -652,13 +652,13 @@
     </row>
     <row r="13">
       <c r="A13" s="5" t="n">
-        <v>46151</v>
+        <v>46212</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="6" t="n"/>
       <c r="E13" s="6" t="n"/>
@@ -666,13 +666,13 @@
     </row>
     <row r="14">
       <c r="A14" s="7" t="n">
-        <v>46152</v>
+        <v>46213</v>
       </c>
       <c r="B14" s="8" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
@@ -680,13 +680,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>46153</v>
+        <v>46214</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D15" s="6" t="n"/>
       <c r="E15" s="6" t="n"/>
@@ -694,13 +694,13 @@
     </row>
     <row r="16">
       <c r="A16" s="7" t="n">
-        <v>46154</v>
+        <v>46215</v>
       </c>
       <c r="B16" s="8" t="n">
         <v>5</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
@@ -708,13 +708,13 @@
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
-        <v>46155</v>
+        <v>46216</v>
       </c>
       <c r="B17" s="6" t="n">
         <v>5</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D17" s="6" t="n"/>
       <c r="E17" s="6" t="n"/>
@@ -722,13 +722,13 @@
     </row>
     <row r="18">
       <c r="A18" s="7" t="n">
-        <v>46156</v>
+        <v>46217</v>
       </c>
       <c r="B18" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="8" t="n"/>
@@ -736,13 +736,13 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>46157</v>
+        <v>46218</v>
       </c>
       <c r="B19" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D19" s="6" t="n"/>
       <c r="E19" s="6" t="n"/>
@@ -750,13 +750,13 @@
     </row>
     <row r="20">
       <c r="A20" s="7" t="n">
-        <v>46158</v>
+        <v>46219</v>
       </c>
       <c r="B20" s="8" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
@@ -764,13 +764,13 @@
     </row>
     <row r="21">
       <c r="A21" s="5" t="n">
-        <v>46159</v>
+        <v>46220</v>
       </c>
       <c r="B21" s="6" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D21" s="6" t="n"/>
       <c r="E21" s="6" t="n"/>
@@ -778,13 +778,13 @@
     </row>
     <row r="22">
       <c r="A22" s="7" t="n">
-        <v>46160</v>
+        <v>46221</v>
       </c>
       <c r="B22" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
@@ -792,10 +792,10 @@
     </row>
     <row r="23">
       <c r="A23" s="5" t="n">
-        <v>46161</v>
+        <v>46222</v>
       </c>
       <c r="B23" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C23" s="6" t="n">
         <v>5</v>
@@ -806,13 +806,13 @@
     </row>
     <row r="24">
       <c r="A24" s="7" t="n">
-        <v>46162</v>
+        <v>46223</v>
       </c>
       <c r="B24" s="8" t="n">
         <v>6</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
@@ -820,10 +820,10 @@
     </row>
     <row r="25">
       <c r="A25" s="5" t="n">
-        <v>46163</v>
+        <v>46224</v>
       </c>
       <c r="B25" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C25" s="6" t="n">
         <v>5</v>
@@ -834,10 +834,10 @@
     </row>
     <row r="26">
       <c r="A26" s="7" t="n">
-        <v>46164</v>
+        <v>46225</v>
       </c>
       <c r="B26" s="8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C26" s="8" t="n">
         <v>5</v>
@@ -848,13 +848,13 @@
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
-        <v>46165</v>
+        <v>46226</v>
       </c>
       <c r="B27" s="6" t="n">
         <v>6</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D27" s="6" t="n"/>
       <c r="E27" s="6" t="n"/>
@@ -862,13 +862,13 @@
     </row>
     <row r="28">
       <c r="A28" s="7" t="n">
-        <v>46166</v>
+        <v>46227</v>
       </c>
       <c r="B28" s="8" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C28" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
@@ -876,13 +876,13 @@
     </row>
     <row r="29">
       <c r="A29" s="5" t="n">
-        <v>46167</v>
+        <v>46228</v>
       </c>
       <c r="B29" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D29" s="6" t="n"/>
       <c r="E29" s="6" t="n"/>
@@ -890,13 +890,13 @@
     </row>
     <row r="30">
       <c r="A30" s="7" t="n">
-        <v>46168</v>
+        <v>46229</v>
       </c>
       <c r="B30" s="8" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
@@ -904,13 +904,13 @@
     </row>
     <row r="31">
       <c r="A31" s="5" t="n">
-        <v>46169</v>
+        <v>46230</v>
       </c>
       <c r="B31" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D31" s="6" t="n"/>
       <c r="E31" s="6" t="n"/>
@@ -918,13 +918,13 @@
     </row>
     <row r="32">
       <c r="A32" s="7" t="n">
-        <v>46170</v>
+        <v>46231</v>
       </c>
       <c r="B32" s="8" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
@@ -932,10 +932,10 @@
     </row>
     <row r="33">
       <c r="A33" s="5" t="n">
-        <v>46171</v>
+        <v>46232</v>
       </c>
       <c r="B33" s="6" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C33" s="6" t="n">
         <v>5</v>
@@ -946,10 +946,10 @@
     </row>
     <row r="34">
       <c r="A34" s="7" t="n">
-        <v>46172</v>
+        <v>46233</v>
       </c>
       <c r="B34" s="8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C34" s="8" t="n">
         <v>4</v>
@@ -960,13 +960,13 @@
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
-        <v>46173</v>
+        <v>46234</v>
       </c>
       <c r="B35" s="6" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D35" s="6" t="n"/>
       <c r="E35" s="6" t="n"/>

</xml_diff>